<commit_message>
Cập nhật dữ liệu campus (Excel) – 23:00:48 27/10/2026
</commit_message>
<xml_diff>
--- a/data/campus-data.xlsx
+++ b/data/campus-data.xlsx
@@ -1,61 +1,107 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EBA047-6ED9-40EE-A60C-D17AE4A851A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="ToaNha" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="CaiDat" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="HuongDan" state="visible" r:id="rId6"/>
+    <sheet name="ToaNha" sheetId="1" r:id="rId1"/>
+    <sheet name="CaiDat" sheetId="2" r:id="rId2"/>
+    <sheet name="HuongDan" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Khớp với khối BLD_&lt;Mã&gt; trong mô hình 3D. Không đổi nếu không đổi mô hình.</t>
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Học tập / Ký túc xá / Thể thao / Cảnh quan / Dịch vụ</t>
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Ngăn cách bằng dấu ;</t>
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Có / Không</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Để trống = không đưa vào tour tự động</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Không xuất ra web</t>
         </r>
       </text>
@@ -65,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="93">
   <si>
     <t>Mã</t>
   </si>
@@ -112,15 +158,9 @@
     <t>A</t>
   </si>
   <si>
-    <t>Tòa A</t>
-  </si>
-  <si>
     <t>Học tập</t>
   </si>
   <si>
-    <t>Tòa tháp trung tâm: sảnh đón, văn phòng tuyển sinh, phòng học</t>
-  </si>
-  <si>
     <t>(cần cập nhật)</t>
   </si>
   <si>
@@ -341,28 +381,40 @@
   </si>
   <si>
     <t>Không đổi tên các sheet và không xóa dòng tiêu đề.</t>
+  </si>
+  <si>
+    <t>Tòa tháp trung tâm: sảnh đón, văn phòng tuyển sinh, phòng học, phòng làm việc CB-GV</t>
+  </si>
+  <si>
+    <t>Tòa Alpha</t>
+  </si>
+  <si>
+    <t>Gồm 13 tầng, tầng 1 để phục vụ Tuyển sinh, tầng 2-9 để dạy học và Hội trường 3 cái ở tầng 5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="14"/>
       <color rgb="FFF37021"/>
-      <sz val="14"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -740,9 +792,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N200"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -757,7 +809,7 @@
     <col min="14" max="14" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -806,652 +858,462 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>90</v>
       </c>
       <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" t="s">
         <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" t="s">
-        <v>20</v>
       </c>
       <c r="M2">
         <v>1</v>
       </c>
       <c r="N2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
       <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" t="s">
         <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L3" t="s">
-        <v>20</v>
       </c>
       <c r="M3">
         <v>2</v>
       </c>
       <c r="N3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" t="s">
         <v>18</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>18</v>
-      </c>
-      <c r="J4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" t="s">
-        <v>19</v>
-      </c>
-      <c r="L4" t="s">
-        <v>20</v>
       </c>
       <c r="M4">
         <v>3</v>
       </c>
       <c r="N4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
       <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" t="s">
         <v>18</v>
-      </c>
-      <c r="H5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L5" t="s">
-        <v>20</v>
       </c>
       <c r="M5">
         <v>5</v>
       </c>
       <c r="N5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
       <c r="G6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" t="s">
         <v>18</v>
-      </c>
-      <c r="H6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" t="s">
-        <v>19</v>
-      </c>
-      <c r="L6" t="s">
-        <v>20</v>
       </c>
       <c r="M6">
         <v>6</v>
       </c>
       <c r="N6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
         <v>34</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>35</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
       <c r="G7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" t="s">
+        <v>17</v>
+      </c>
+      <c r="L7" t="s">
         <v>18</v>
-      </c>
-      <c r="H7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L7" t="s">
-        <v>20</v>
       </c>
       <c r="M7">
         <v>7</v>
       </c>
       <c r="N7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
         <v>38</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
       <c r="G8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" t="s">
         <v>18</v>
-      </c>
-      <c r="H8" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" t="s">
-        <v>19</v>
-      </c>
-      <c r="L8" t="s">
-        <v>20</v>
       </c>
       <c r="M8">
         <v>4</v>
       </c>
       <c r="N8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
         <v>42</v>
       </c>
-      <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" t="s">
-        <v>44</v>
-      </c>
       <c r="G9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" t="s">
         <v>18</v>
-      </c>
-      <c r="H9" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" t="s">
-        <v>19</v>
-      </c>
-      <c r="L9" t="s">
-        <v>20</v>
       </c>
       <c r="M9">
         <v>8</v>
       </c>
       <c r="N9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
         <v>45</v>
       </c>
-      <c r="B10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
       <c r="G10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L10" t="s">
         <v>18</v>
       </c>
-      <c r="H10" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="N10" t="s">
         <v>19</v>
-      </c>
-      <c r="K10" t="s">
-        <v>19</v>
-      </c>
-      <c r="L10" t="s">
-        <v>20</v>
-      </c>
-      <c r="N10" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" t="s">
         <v>48</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
       <c r="G11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" t="s">
+        <v>17</v>
+      </c>
+      <c r="L11" t="s">
         <v>18</v>
       </c>
-      <c r="H11" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="N11" t="s">
         <v>19</v>
-      </c>
-      <c r="K11" t="s">
-        <v>19</v>
-      </c>
-      <c r="L11" t="s">
-        <v>20</v>
-      </c>
-      <c r="N11" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" t="s">
         <v>52</v>
       </c>
-      <c r="B12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" t="s">
-        <v>54</v>
-      </c>
       <c r="G12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" t="s">
+        <v>17</v>
+      </c>
+      <c r="K12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L12" t="s">
         <v>18</v>
       </c>
-      <c r="H12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I12" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="N12" t="s">
         <v>19</v>
-      </c>
-      <c r="K12" t="s">
-        <v>19</v>
-      </c>
-      <c r="L12" t="s">
-        <v>20</v>
-      </c>
-      <c r="N12" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
         <v>55</v>
       </c>
-      <c r="B13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" t="s">
-        <v>57</v>
-      </c>
       <c r="G13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" t="s">
+        <v>17</v>
+      </c>
+      <c r="K13" t="s">
+        <v>17</v>
+      </c>
+      <c r="L13" t="s">
         <v>18</v>
       </c>
-      <c r="H13" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="N13" t="s">
         <v>19</v>
       </c>
-      <c r="K13" t="s">
-        <v>19</v>
-      </c>
-      <c r="L13" t="s">
-        <v>20</v>
-      </c>
-      <c r="N13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="12:12" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="12:12" x14ac:dyDescent="0.25"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="L10:L200">
-      <formula1>"Có,Không"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L2:L200">
+  <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="L2:L200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Có,Không"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="3" width="45" customWidth="1"/>
@@ -1459,169 +1321,169 @@
   <sheetData>
     <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
         <v>61</v>
-      </c>
-      <c r="B2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" t="s">
         <v>64</v>
-      </c>
-      <c r="B3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" t="s">
         <v>67</v>
-      </c>
-      <c r="B4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
         <v>70</v>
-      </c>
-      <c r="B5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
         <v>73</v>
-      </c>
-      <c r="B6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" t="s">
         <v>76</v>
-      </c>
-      <c r="B7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C7" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s">
         <v>81</v>
-      </c>
-      <c r="B9" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" t="s">
-        <v>83</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>